<commit_message>
UX decks: approval steps named by their action in the swimlanes, whole windows on one slide, long titles in a smaller type, menus four columns wide; the UX state of the refused and confirmed walkthrough steps; UX documents of the three Drop 0 sets rebuilt
</commit_message>
<xml_diff>
--- a/docs/deliverables/out/Drop-0_Setup_and_Data_Migration/BRD-03_Product_Maintenance/08_BIBS_UXScreens_BRD-03_Product_Maintenance_v2.0.xlsx
+++ b/docs/deliverables/out/Drop-0_Setup_and_Data_Migration/BRD-03_Product_Maintenance/08_BIBS_UXScreens_BRD-03_Product_Maintenance_v2.0.xlsx
@@ -7233,7 +7233,7 @@
       </c>
       <c r="G99" s="45" t="inlineStr">
         <is>
-          <t>Success message</t>
+          <t>Validation error</t>
         </is>
       </c>
       <c r="H99" s="45" t="inlineStr">
@@ -7357,7 +7357,7 @@
       </c>
       <c r="G101" s="45" t="inlineStr">
         <is>
-          <t>Success message</t>
+          <t>Validation error</t>
         </is>
       </c>
       <c r="H101" s="45" t="inlineStr">

</xml_diff>

<commit_message>
BRD-03 Product Maintenance screenshots retaken in the BDO style-guide presentation on a fresh seed stack: 126 images; FRS, guide deck, sign-off workbook and UX documents 07 to 09 rebuilt at v2.0 with issue 2.2 change CHG-PM-2.2-01; insurer responses described with their row action menu; capture opens a row action when the button is in the menu
</commit_message>
<xml_diff>
--- a/docs/deliverables/out/Drop-0_Setup_and_Data_Migration/BRD-03_Product_Maintenance/08_BIBS_UXScreens_BRD-03_Product_Maintenance_v2.0.xlsx
+++ b/docs/deliverables/out/Drop-0_Setup_and_Data_Migration/BRD-03_Product_Maintenance/08_BIBS_UXScreens_BRD-03_Product_Maintenance_v2.0.xlsx
@@ -689,7 +689,7 @@
 Mandatory: Yes
 Format: Y or N
 Allowed values: Y or N
-Example: N</t>
+Example: Y</t>
       </text>
     </comment>
     <comment ref="O16" authorId="0" shapeId="0">
@@ -698,7 +698,8 @@
 The change reference (comment, change request or issue change) that changed the image
 Mandatory: Conditional: when Changed in this issue is Y
 Format: Reference
-Allowed values: Free entry</t>
+Allowed values: Free entry
+Example: CHG-PM-2.2-01</t>
       </text>
     </comment>
   </commentList>
@@ -1073,7 +1074,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A2:I37"/>
+  <dimension ref="A2:I38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1348,7 +1349,7 @@
       </c>
       <c r="D22" s="14" t="inlineStr">
         <is>
-          <t>123 screen images of 39 screens; 19 changed in this issue</t>
+          <t>123 screen images of 39 screens; 95 changed in this issue</t>
         </is>
       </c>
       <c r="E22" s="14" t="inlineStr">
@@ -1520,43 +1521,47 @@
       </c>
       <c r="I30" s="5" t="n"/>
     </row>
-    <row r="32">
-      <c r="A32" s="8" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="14" t="inlineStr">
+        <is>
+          <t>CHG-PM-2.2-01</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n"/>
+      <c r="C31" s="14" t="inlineStr">
+        <is>
+          <t>Lists in the BDO style guide: outlined status pills, alternating white and Background Blue rows, a long list scrolling inside its card with the header row in view, names instead of codes, due dates on one line with the overdue icon and ages in words; every image of the set retaken</t>
+        </is>
+      </c>
+      <c r="D31" s="18" t="n"/>
+      <c r="E31" s="18" t="n"/>
+      <c r="F31" s="18" t="n"/>
+      <c r="G31" s="5" t="n"/>
+      <c r="H31" s="14" t="inlineStr">
+        <is>
+          <t>SCR-PM-01, SCR-PM-02, SCR-PM-03, SCR-PM-04, SCR-PM-05, SCR-PM-06, SCR-PM-07, SCR-PM-08, SCR-PM-09, SCR-PM-10, SCR-PM-11, SCR-PM-12, SCR-PM-13, SCR-PM-14, SCR-PM-15, SCR-PM-16, SCR-PM-17, SCR-PM-18, SCR-PM-19, SCR-PM-20, SCR-PM-21, SCR-PM-22</t>
+        </is>
+      </c>
+      <c r="I31" s="5" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="8" t="inlineStr">
         <is>
           <t>Other sheets</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="17" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="17" t="inlineStr">
         <is>
           <t>Sheet</t>
-        </is>
-      </c>
-      <c r="B33" s="18" t="n"/>
-      <c r="C33" s="5" t="n"/>
-      <c r="D33" s="17" t="inlineStr">
-        <is>
-          <t>What it holds</t>
-        </is>
-      </c>
-      <c r="E33" s="18" t="n"/>
-      <c r="F33" s="18" t="n"/>
-      <c r="G33" s="18" t="n"/>
-      <c r="H33" s="18" t="n"/>
-      <c r="I33" s="5" t="n"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="16" t="inlineStr">
-        <is>
-          <t>Reference lists</t>
         </is>
       </c>
       <c r="B34" s="18" t="n"/>
       <c r="C34" s="5" t="n"/>
-      <c r="D34" s="14" t="inlineStr">
-        <is>
-          <t>The lists of the drop-downs: states and UXD statuses</t>
+      <c r="D34" s="17" t="inlineStr">
+        <is>
+          <t>What it holds</t>
         </is>
       </c>
       <c r="E34" s="18" t="n"/>
@@ -1568,14 +1573,14 @@
     <row r="35">
       <c r="A35" s="16" t="inlineStr">
         <is>
-          <t>Questions and comments</t>
+          <t>Reference lists</t>
         </is>
       </c>
       <c r="B35" s="18" t="n"/>
       <c r="C35" s="5" t="n"/>
       <c r="D35" s="14" t="inlineStr">
         <is>
-          <t>Questions and comments of the UX Design team, with the answer</t>
+          <t>The lists of the drop-downs: states and UXD statuses</t>
         </is>
       </c>
       <c r="E35" s="18" t="n"/>
@@ -1584,8 +1589,27 @@
       <c r="H35" s="18" t="n"/>
       <c r="I35" s="5" t="n"/>
     </row>
-    <row r="37">
-      <c r="A37" s="19" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="16" t="inlineStr">
+        <is>
+          <t>Questions and comments</t>
+        </is>
+      </c>
+      <c r="B36" s="18" t="n"/>
+      <c r="C36" s="5" t="n"/>
+      <c r="D36" s="14" t="inlineStr">
+        <is>
+          <t>Questions and comments of the UX Design team, with the answer</t>
+        </is>
+      </c>
+      <c r="E36" s="18" t="n"/>
+      <c r="F36" s="18" t="n"/>
+      <c r="G36" s="18" t="n"/>
+      <c r="H36" s="18" t="n"/>
+      <c r="I36" s="5" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="19" t="inlineStr">
         <is>
           <t>Prepared by iorta TechNXT for BDOI. Confidential – BDOI.</t>
         </is>
@@ -1593,7 +1617,7 @@
     </row>
   </sheetData>
   <autoFilter ref="A21:I22"/>
-  <mergeCells count="41">
+  <mergeCells count="44">
     <mergeCell ref="C10:H10"/>
     <mergeCell ref="A30:B30"/>
     <mergeCell ref="C30:G30"/>
@@ -1601,23 +1625,23 @@
     <mergeCell ref="A11:B11"/>
     <mergeCell ref="C9:H9"/>
     <mergeCell ref="B16:I16"/>
+    <mergeCell ref="H31:I31"/>
     <mergeCell ref="A6:B6"/>
     <mergeCell ref="C26:G26"/>
     <mergeCell ref="B18:I18"/>
     <mergeCell ref="C11:H11"/>
     <mergeCell ref="H25:I25"/>
     <mergeCell ref="C29:G29"/>
-    <mergeCell ref="A33:C33"/>
     <mergeCell ref="A7:B7"/>
     <mergeCell ref="A25:B25"/>
     <mergeCell ref="C25:G25"/>
     <mergeCell ref="C8:H8"/>
     <mergeCell ref="B14:I14"/>
+    <mergeCell ref="C31:G31"/>
     <mergeCell ref="A35:C35"/>
     <mergeCell ref="A27:B27"/>
     <mergeCell ref="C7:H7"/>
     <mergeCell ref="B17:I17"/>
-    <mergeCell ref="D33:I33"/>
     <mergeCell ref="A26:B26"/>
     <mergeCell ref="C27:G27"/>
     <mergeCell ref="D35:I35"/>
@@ -1627,12 +1651,15 @@
     <mergeCell ref="H27:I27"/>
     <mergeCell ref="D34:I34"/>
     <mergeCell ref="C6:H6"/>
+    <mergeCell ref="A36:C36"/>
     <mergeCell ref="A29:B29"/>
     <mergeCell ref="B15:I15"/>
     <mergeCell ref="A10:B10"/>
     <mergeCell ref="A28:B28"/>
     <mergeCell ref="C28:G28"/>
+    <mergeCell ref="D36:I36"/>
     <mergeCell ref="A9:B9"/>
+    <mergeCell ref="A31:B31"/>
     <mergeCell ref="H30:I30"/>
     <mergeCell ref="H26:I26"/>
   </mergeCells>
@@ -1662,8 +1689,8 @@
   </dataValidations>
   <hyperlinks>
     <hyperlink ref="I22" location="'UX screen register'!A1"/>
-    <hyperlink ref="A34" location="'Reference lists'!A1"/>
-    <hyperlink ref="A35" location="'Questions and comments'!A1"/>
+    <hyperlink ref="A35" location="'Reference lists'!A1"/>
+    <hyperlink ref="A36" location="'Questions and comments'!A1"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.4" right="0.4" top="0.6" bottom="0.6" header="0.5" footer="0.5"/>
@@ -2306,10 +2333,14 @@
       <c r="M17" s="43" t="n"/>
       <c r="N17" s="43" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O17" s="43" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O17" s="43" t="inlineStr">
+        <is>
+          <t>CHG-PM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="B18" s="45" t="inlineStr">
@@ -2366,10 +2397,14 @@
       <c r="M18" s="45" t="n"/>
       <c r="N18" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O18" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O18" s="45" t="inlineStr">
+        <is>
+          <t>CHG-PM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="B19" s="45" t="inlineStr">
@@ -2426,10 +2461,14 @@
       <c r="M19" s="45" t="n"/>
       <c r="N19" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O19" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O19" s="45" t="inlineStr">
+        <is>
+          <t>CHG-PM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="B20" s="45" t="inlineStr">
@@ -2486,10 +2525,14 @@
       <c r="M20" s="45" t="n"/>
       <c r="N20" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O20" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O20" s="45" t="inlineStr">
+        <is>
+          <t>CHG-PM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="B21" s="45" t="inlineStr">
@@ -2551,7 +2594,7 @@
       </c>
       <c r="O21" s="45" t="inlineStr">
         <is>
-          <t>CHG-PM-2.1-03</t>
+          <t>CHG-PM-2.1-03, CHG-PM-2.2-01</t>
         </is>
       </c>
     </row>
@@ -2615,7 +2658,7 @@
       </c>
       <c r="O22" s="45" t="inlineStr">
         <is>
-          <t>CHG-PM-2.1-03</t>
+          <t>CHG-PM-2.1-03, CHG-PM-2.2-01</t>
         </is>
       </c>
     </row>
@@ -2679,7 +2722,7 @@
       </c>
       <c r="O23" s="45" t="inlineStr">
         <is>
-          <t>CHG-PM-2.1-03</t>
+          <t>CHG-PM-2.1-03, CHG-PM-2.2-01</t>
         </is>
       </c>
     </row>
@@ -2743,7 +2786,7 @@
       </c>
       <c r="O24" s="45" t="inlineStr">
         <is>
-          <t>CHG-PM-2.1-04</t>
+          <t>CHG-PM-2.1-04, CHG-PM-2.2-01</t>
         </is>
       </c>
     </row>
@@ -2807,7 +2850,7 @@
       </c>
       <c r="O25" s="45" t="inlineStr">
         <is>
-          <t>CHG-PM-2.1-04</t>
+          <t>CHG-PM-2.1-04, CHG-PM-2.2-01</t>
         </is>
       </c>
     </row>
@@ -2866,10 +2909,14 @@
       <c r="M26" s="45" t="n"/>
       <c r="N26" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O26" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O26" s="45" t="inlineStr">
+        <is>
+          <t>CHG-PM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="B27" s="45" t="inlineStr">
@@ -2926,10 +2973,14 @@
       <c r="M27" s="45" t="n"/>
       <c r="N27" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O27" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O27" s="45" t="inlineStr">
+        <is>
+          <t>CHG-PM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="B28" s="45" t="inlineStr">
@@ -2991,7 +3042,7 @@
       </c>
       <c r="O28" s="45" t="inlineStr">
         <is>
-          <t>CHG-PM-2.1-04</t>
+          <t>CHG-PM-2.1-04, CHG-PM-2.2-01</t>
         </is>
       </c>
     </row>
@@ -3050,10 +3101,14 @@
       <c r="M29" s="45" t="n"/>
       <c r="N29" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O29" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O29" s="45" t="inlineStr">
+        <is>
+          <t>CHG-PM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="B30" s="45" t="inlineStr">
@@ -3110,10 +3165,14 @@
       <c r="M30" s="45" t="n"/>
       <c r="N30" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O30" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O30" s="45" t="inlineStr">
+        <is>
+          <t>CHG-PM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="B31" s="45" t="inlineStr">
@@ -3170,10 +3229,14 @@
       <c r="M31" s="45" t="n"/>
       <c r="N31" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O31" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O31" s="45" t="inlineStr">
+        <is>
+          <t>CHG-PM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="B32" s="45" t="inlineStr">
@@ -3230,10 +3293,14 @@
       <c r="M32" s="45" t="n"/>
       <c r="N32" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O32" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O32" s="45" t="inlineStr">
+        <is>
+          <t>CHG-PM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="B33" s="45" t="inlineStr">
@@ -3290,10 +3357,14 @@
       <c r="M33" s="45" t="n"/>
       <c r="N33" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O33" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O33" s="45" t="inlineStr">
+        <is>
+          <t>CHG-PM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="B34" s="45" t="inlineStr">
@@ -3350,10 +3421,14 @@
       <c r="M34" s="45" t="n"/>
       <c r="N34" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O34" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O34" s="45" t="inlineStr">
+        <is>
+          <t>CHG-PM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="B35" s="45" t="inlineStr">
@@ -3410,10 +3485,14 @@
       <c r="M35" s="45" t="n"/>
       <c r="N35" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O35" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O35" s="45" t="inlineStr">
+        <is>
+          <t>CHG-PM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="B36" s="45" t="inlineStr">
@@ -3470,10 +3549,14 @@
       <c r="M36" s="45" t="n"/>
       <c r="N36" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O36" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O36" s="45" t="inlineStr">
+        <is>
+          <t>CHG-PM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="B37" s="45" t="inlineStr">
@@ -3530,10 +3613,14 @@
       <c r="M37" s="45" t="n"/>
       <c r="N37" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O37" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O37" s="45" t="inlineStr">
+        <is>
+          <t>CHG-PM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="B38" s="45" t="inlineStr">
@@ -3590,10 +3677,14 @@
       <c r="M38" s="45" t="n"/>
       <c r="N38" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O38" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O38" s="45" t="inlineStr">
+        <is>
+          <t>CHG-PM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="B39" s="45" t="inlineStr">
@@ -3650,10 +3741,14 @@
       <c r="M39" s="45" t="n"/>
       <c r="N39" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O39" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O39" s="45" t="inlineStr">
+        <is>
+          <t>CHG-PM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="B40" s="45" t="inlineStr">
@@ -3710,10 +3805,14 @@
       <c r="M40" s="45" t="n"/>
       <c r="N40" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O40" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O40" s="45" t="inlineStr">
+        <is>
+          <t>CHG-PM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="B41" s="45" t="inlineStr">
@@ -3770,10 +3869,14 @@
       <c r="M41" s="45" t="n"/>
       <c r="N41" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O41" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O41" s="45" t="inlineStr">
+        <is>
+          <t>CHG-PM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="B42" s="45" t="inlineStr">
@@ -3835,7 +3938,7 @@
       </c>
       <c r="O42" s="45" t="inlineStr">
         <is>
-          <t>CHG-PM-2.1-05</t>
+          <t>CHG-PM-2.1-05, CHG-PM-2.2-01</t>
         </is>
       </c>
     </row>
@@ -3894,10 +3997,14 @@
       <c r="M43" s="45" t="n"/>
       <c r="N43" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O43" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O43" s="45" t="inlineStr">
+        <is>
+          <t>CHG-PM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="B44" s="45" t="inlineStr">
@@ -3954,10 +4061,14 @@
       <c r="M44" s="45" t="n"/>
       <c r="N44" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O44" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O44" s="45" t="inlineStr">
+        <is>
+          <t>CHG-PM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="B45" s="45" t="inlineStr">
@@ -4019,7 +4130,7 @@
       </c>
       <c r="O45" s="45" t="inlineStr">
         <is>
-          <t>CHG-PM-2.1-05</t>
+          <t>CHG-PM-2.1-05, CHG-PM-2.2-01</t>
         </is>
       </c>
     </row>
@@ -4078,10 +4189,14 @@
       <c r="M46" s="45" t="n"/>
       <c r="N46" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O46" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O46" s="45" t="inlineStr">
+        <is>
+          <t>CHG-PM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="B47" s="45" t="inlineStr">
@@ -4138,10 +4253,14 @@
       <c r="M47" s="45" t="n"/>
       <c r="N47" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O47" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O47" s="45" t="inlineStr">
+        <is>
+          <t>CHG-PM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="B48" s="45" t="inlineStr">
@@ -4198,10 +4317,14 @@
       <c r="M48" s="45" t="n"/>
       <c r="N48" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O48" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O48" s="45" t="inlineStr">
+        <is>
+          <t>CHG-PM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="B49" s="45" t="inlineStr">
@@ -4258,10 +4381,14 @@
       <c r="M49" s="45" t="n"/>
       <c r="N49" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O49" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O49" s="45" t="inlineStr">
+        <is>
+          <t>CHG-PM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="B50" s="45" t="inlineStr">
@@ -4318,10 +4445,14 @@
       <c r="M50" s="45" t="n"/>
       <c r="N50" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O50" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O50" s="45" t="inlineStr">
+        <is>
+          <t>CHG-PM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="B51" s="45" t="inlineStr">
@@ -4378,10 +4509,14 @@
       <c r="M51" s="45" t="n"/>
       <c r="N51" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O51" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O51" s="45" t="inlineStr">
+        <is>
+          <t>CHG-PM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="B52" s="45" t="inlineStr">
@@ -4443,7 +4578,7 @@
       </c>
       <c r="O52" s="45" t="inlineStr">
         <is>
-          <t>CHG-PM-2.1-01</t>
+          <t>CHG-PM-2.1-01, CHG-PM-2.2-01</t>
         </is>
       </c>
     </row>
@@ -4507,7 +4642,7 @@
       </c>
       <c r="O53" s="45" t="inlineStr">
         <is>
-          <t>CHG-PM-2.1-01, CHG-PM-2.1-02</t>
+          <t>CHG-PM-2.1-01, CHG-PM-2.1-02, CHG-PM-2.2-01</t>
         </is>
       </c>
     </row>
@@ -4566,10 +4701,14 @@
       <c r="M54" s="45" t="n"/>
       <c r="N54" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O54" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O54" s="45" t="inlineStr">
+        <is>
+          <t>CHG-PM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="B55" s="45" t="inlineStr">
@@ -4631,7 +4770,7 @@
       </c>
       <c r="O55" s="45" t="inlineStr">
         <is>
-          <t>CHG-PM-2.1-05</t>
+          <t>CHG-PM-2.1-05, CHG-PM-2.2-01</t>
         </is>
       </c>
     </row>
@@ -4695,7 +4834,7 @@
       </c>
       <c r="O56" s="45" t="inlineStr">
         <is>
-          <t>CHG-PM-2.1-05</t>
+          <t>CHG-PM-2.1-05, CHG-PM-2.2-01</t>
         </is>
       </c>
     </row>
@@ -4754,10 +4893,14 @@
       <c r="M57" s="45" t="n"/>
       <c r="N57" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O57" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O57" s="45" t="inlineStr">
+        <is>
+          <t>CHG-PM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="B58" s="45" t="inlineStr">
@@ -4819,7 +4962,7 @@
       </c>
       <c r="O58" s="45" t="inlineStr">
         <is>
-          <t>CHG-PM-2.1-05</t>
+          <t>CHG-PM-2.1-05, CHG-PM-2.2-01</t>
         </is>
       </c>
     </row>
@@ -4878,10 +5021,14 @@
       <c r="M59" s="45" t="n"/>
       <c r="N59" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O59" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O59" s="45" t="inlineStr">
+        <is>
+          <t>CHG-PM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="B60" s="45" t="inlineStr">
@@ -4943,7 +5090,7 @@
       </c>
       <c r="O60" s="45" t="inlineStr">
         <is>
-          <t>CHG-PM-2.1-05</t>
+          <t>CHG-PM-2.1-05, CHG-PM-2.2-01</t>
         </is>
       </c>
     </row>
@@ -5002,10 +5149,14 @@
       <c r="M61" s="45" t="n"/>
       <c r="N61" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O61" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O61" s="45" t="inlineStr">
+        <is>
+          <t>CHG-PM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="B62" s="45" t="inlineStr">
@@ -5067,7 +5218,7 @@
       </c>
       <c r="O62" s="45" t="inlineStr">
         <is>
-          <t>CHG-PM-2.1-05</t>
+          <t>CHG-PM-2.1-05, CHG-PM-2.2-01</t>
         </is>
       </c>
     </row>
@@ -5131,7 +5282,7 @@
       </c>
       <c r="O63" s="45" t="inlineStr">
         <is>
-          <t>CHG-PM-2.1-05</t>
+          <t>CHG-PM-2.1-05, CHG-PM-2.2-01</t>
         </is>
       </c>
     </row>
@@ -5190,10 +5341,14 @@
       <c r="M64" s="45" t="n"/>
       <c r="N64" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O64" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O64" s="45" t="inlineStr">
+        <is>
+          <t>CHG-PM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="B65" s="45" t="inlineStr">
@@ -5250,10 +5405,14 @@
       <c r="M65" s="45" t="n"/>
       <c r="N65" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O65" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O65" s="45" t="inlineStr">
+        <is>
+          <t>CHG-PM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="B66" s="45" t="inlineStr">
@@ -5310,10 +5469,14 @@
       <c r="M66" s="45" t="n"/>
       <c r="N66" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O66" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O66" s="45" t="inlineStr">
+        <is>
+          <t>CHG-PM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="B67" s="45" t="inlineStr">
@@ -5370,10 +5533,14 @@
       <c r="M67" s="45" t="n"/>
       <c r="N67" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O67" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O67" s="45" t="inlineStr">
+        <is>
+          <t>CHG-PM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="B68" s="45" t="inlineStr">
@@ -5430,10 +5597,14 @@
       <c r="M68" s="45" t="n"/>
       <c r="N68" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O68" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O68" s="45" t="inlineStr">
+        <is>
+          <t>CHG-PM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="B69" s="45" t="inlineStr">
@@ -5490,10 +5661,14 @@
       <c r="M69" s="45" t="n"/>
       <c r="N69" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O69" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O69" s="45" t="inlineStr">
+        <is>
+          <t>CHG-PM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="B70" s="45" t="inlineStr">
@@ -5550,10 +5725,14 @@
       <c r="M70" s="45" t="n"/>
       <c r="N70" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O70" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O70" s="45" t="inlineStr">
+        <is>
+          <t>CHG-PM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="B71" s="45" t="inlineStr">
@@ -5610,10 +5789,14 @@
       <c r="M71" s="45" t="n"/>
       <c r="N71" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O71" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O71" s="45" t="inlineStr">
+        <is>
+          <t>CHG-PM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="B72" s="45" t="inlineStr">
@@ -5670,10 +5853,14 @@
       <c r="M72" s="45" t="n"/>
       <c r="N72" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O72" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O72" s="45" t="inlineStr">
+        <is>
+          <t>CHG-PM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="B73" s="45" t="inlineStr">
@@ -5732,10 +5919,14 @@
       <c r="M73" s="45" t="n"/>
       <c r="N73" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O73" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O73" s="45" t="inlineStr">
+        <is>
+          <t>CHG-PM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="B74" s="45" t="inlineStr">
@@ -5794,10 +5985,14 @@
       <c r="M74" s="45" t="n"/>
       <c r="N74" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O74" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O74" s="45" t="inlineStr">
+        <is>
+          <t>CHG-PM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="B75" s="45" t="inlineStr">
@@ -5856,10 +6051,14 @@
       <c r="M75" s="45" t="n"/>
       <c r="N75" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O75" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O75" s="45" t="inlineStr">
+        <is>
+          <t>CHG-PM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="B76" s="45" t="inlineStr">
@@ -5918,10 +6117,14 @@
       <c r="M76" s="45" t="n"/>
       <c r="N76" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O76" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O76" s="45" t="inlineStr">
+        <is>
+          <t>CHG-PM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="B77" s="45" t="inlineStr">
@@ -5980,10 +6183,14 @@
       <c r="M77" s="45" t="n"/>
       <c r="N77" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O77" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O77" s="45" t="inlineStr">
+        <is>
+          <t>CHG-PM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="B78" s="45" t="inlineStr">
@@ -6042,10 +6249,14 @@
       <c r="M78" s="45" t="n"/>
       <c r="N78" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O78" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O78" s="45" t="inlineStr">
+        <is>
+          <t>CHG-PM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="B79" s="45" t="inlineStr">
@@ -6104,10 +6315,14 @@
       <c r="M79" s="45" t="n"/>
       <c r="N79" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O79" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O79" s="45" t="inlineStr">
+        <is>
+          <t>CHG-PM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="B80" s="45" t="inlineStr">
@@ -6166,10 +6381,14 @@
       <c r="M80" s="45" t="n"/>
       <c r="N80" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O80" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O80" s="45" t="inlineStr">
+        <is>
+          <t>CHG-PM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="B81" s="45" t="inlineStr">
@@ -6228,10 +6447,14 @@
       <c r="M81" s="45" t="n"/>
       <c r="N81" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O81" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O81" s="45" t="inlineStr">
+        <is>
+          <t>CHG-PM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="B82" s="45" t="inlineStr">
@@ -6290,10 +6513,14 @@
       <c r="M82" s="45" t="n"/>
       <c r="N82" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O82" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O82" s="45" t="inlineStr">
+        <is>
+          <t>CHG-PM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="B83" s="45" t="inlineStr">
@@ -6352,10 +6579,14 @@
       <c r="M83" s="45" t="n"/>
       <c r="N83" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O83" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O83" s="45" t="inlineStr">
+        <is>
+          <t>CHG-PM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="B84" s="45" t="inlineStr">
@@ -6414,10 +6645,14 @@
       <c r="M84" s="45" t="n"/>
       <c r="N84" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O84" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O84" s="45" t="inlineStr">
+        <is>
+          <t>CHG-PM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="B85" s="45" t="inlineStr">
@@ -6476,10 +6711,14 @@
       <c r="M85" s="45" t="n"/>
       <c r="N85" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O85" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O85" s="45" t="inlineStr">
+        <is>
+          <t>CHG-PM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="B86" s="45" t="inlineStr">
@@ -6538,10 +6777,14 @@
       <c r="M86" s="45" t="n"/>
       <c r="N86" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O86" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O86" s="45" t="inlineStr">
+        <is>
+          <t>CHG-PM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="B87" s="45" t="inlineStr">
@@ -6600,10 +6843,14 @@
       <c r="M87" s="45" t="n"/>
       <c r="N87" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O87" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O87" s="45" t="inlineStr">
+        <is>
+          <t>CHG-PM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="B88" s="45" t="inlineStr">
@@ -6667,7 +6914,7 @@
       </c>
       <c r="O88" s="45" t="inlineStr">
         <is>
-          <t>CHG-PM-2.1-01</t>
+          <t>CHG-PM-2.1-01, CHG-PM-2.2-01</t>
         </is>
       </c>
     </row>
@@ -6733,7 +6980,7 @@
       </c>
       <c r="O89" s="45" t="inlineStr">
         <is>
-          <t>CHG-PM-2.1-01, CHG-PM-2.1-02</t>
+          <t>CHG-PM-2.1-01, CHG-PM-2.1-02, CHG-PM-2.2-01</t>
         </is>
       </c>
     </row>
@@ -6794,10 +7041,14 @@
       <c r="M90" s="45" t="n"/>
       <c r="N90" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O90" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O90" s="45" t="inlineStr">
+        <is>
+          <t>CHG-PM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="B91" s="45" t="inlineStr">
@@ -6856,10 +7107,14 @@
       <c r="M91" s="45" t="n"/>
       <c r="N91" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O91" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O91" s="45" t="inlineStr">
+        <is>
+          <t>CHG-PM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="B92" s="45" t="inlineStr">
@@ -6918,10 +7173,14 @@
       <c r="M92" s="45" t="n"/>
       <c r="N92" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O92" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O92" s="45" t="inlineStr">
+        <is>
+          <t>CHG-PM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="B93" s="45" t="inlineStr">
@@ -6980,10 +7239,14 @@
       <c r="M93" s="45" t="n"/>
       <c r="N93" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O93" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O93" s="45" t="inlineStr">
+        <is>
+          <t>CHG-PM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="B94" s="45" t="inlineStr">
@@ -7042,10 +7305,14 @@
       <c r="M94" s="45" t="n"/>
       <c r="N94" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O94" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O94" s="45" t="inlineStr">
+        <is>
+          <t>CHG-PM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="B95" s="45" t="inlineStr">
@@ -7104,10 +7371,14 @@
       <c r="M95" s="45" t="n"/>
       <c r="N95" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O95" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O95" s="45" t="inlineStr">
+        <is>
+          <t>CHG-PM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="B96" s="45" t="inlineStr">
@@ -7166,10 +7437,14 @@
       <c r="M96" s="45" t="n"/>
       <c r="N96" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O96" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O96" s="45" t="inlineStr">
+        <is>
+          <t>CHG-PM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="B97" s="45" t="inlineStr">
@@ -7228,10 +7503,14 @@
       <c r="M97" s="45" t="n"/>
       <c r="N97" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O97" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O97" s="45" t="inlineStr">
+        <is>
+          <t>CHG-PM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="B98" s="45" t="inlineStr">
@@ -7290,10 +7569,14 @@
       <c r="M98" s="45" t="n"/>
       <c r="N98" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O98" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O98" s="45" t="inlineStr">
+        <is>
+          <t>CHG-PM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="B99" s="45" t="inlineStr">
@@ -7352,10 +7635,14 @@
       <c r="M99" s="45" t="n"/>
       <c r="N99" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O99" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O99" s="45" t="inlineStr">
+        <is>
+          <t>CHG-PM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="B100" s="45" t="inlineStr">
@@ -7414,10 +7701,14 @@
       <c r="M100" s="45" t="n"/>
       <c r="N100" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O100" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O100" s="45" t="inlineStr">
+        <is>
+          <t>CHG-PM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="B101" s="45" t="inlineStr">
@@ -7476,10 +7767,14 @@
       <c r="M101" s="45" t="n"/>
       <c r="N101" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O101" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O101" s="45" t="inlineStr">
+        <is>
+          <t>CHG-PM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="B102" s="45" t="inlineStr">
@@ -7538,10 +7833,14 @@
       <c r="M102" s="45" t="n"/>
       <c r="N102" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O102" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O102" s="45" t="inlineStr">
+        <is>
+          <t>CHG-PM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="B103" s="45" t="inlineStr">
@@ -7600,10 +7899,14 @@
       <c r="M103" s="45" t="n"/>
       <c r="N103" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O103" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O103" s="45" t="inlineStr">
+        <is>
+          <t>CHG-PM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="B104" s="45" t="inlineStr">
@@ -7662,10 +7965,14 @@
       <c r="M104" s="45" t="n"/>
       <c r="N104" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O104" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O104" s="45" t="inlineStr">
+        <is>
+          <t>CHG-PM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="B105" s="45" t="inlineStr">
@@ -7724,10 +8031,14 @@
       <c r="M105" s="45" t="n"/>
       <c r="N105" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O105" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O105" s="45" t="inlineStr">
+        <is>
+          <t>CHG-PM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="B106" s="45" t="inlineStr">
@@ -7786,10 +8097,14 @@
       <c r="M106" s="45" t="n"/>
       <c r="N106" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O106" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O106" s="45" t="inlineStr">
+        <is>
+          <t>CHG-PM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="B107" s="45" t="inlineStr">
@@ -7848,10 +8163,14 @@
       <c r="M107" s="45" t="n"/>
       <c r="N107" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O107" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O107" s="45" t="inlineStr">
+        <is>
+          <t>CHG-PM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="B108" s="45" t="inlineStr">
@@ -7910,10 +8229,14 @@
       <c r="M108" s="45" t="n"/>
       <c r="N108" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O108" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O108" s="45" t="inlineStr">
+        <is>
+          <t>CHG-PM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="B109" s="45" t="inlineStr">
@@ -9650,10 +9973,14 @@
       <c r="M137" s="45" t="n"/>
       <c r="N137" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O137" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O137" s="45" t="inlineStr">
+        <is>
+          <t>CHG-PM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="B138" s="45" t="inlineStr">
@@ -9715,7 +10042,7 @@
       </c>
       <c r="O138" s="45" t="inlineStr">
         <is>
-          <t>CHG-PM-2.1-03</t>
+          <t>CHG-PM-2.1-03, CHG-PM-2.2-01</t>
         </is>
       </c>
     </row>
@@ -9774,10 +10101,14 @@
       <c r="M139" s="45" t="n"/>
       <c r="N139" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O139" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O139" s="45" t="inlineStr">
+        <is>
+          <t>CHG-PM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="B140" s="45" t="inlineStr">
@@ -9834,10 +10165,14 @@
       <c r="M140" s="45" t="n"/>
       <c r="N140" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O140" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O140" s="45" t="inlineStr">
+        <is>
+          <t>CHG-PM-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="B141" s="46" t="n"/>

</xml_diff>